<commit_message>
Button BOM minor fix #23
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Button-v1.2/BOM/eSpark-BOM-IoT-Button.xlsx
+++ b/Design Files/IoT-Button-v1.2/BOM/eSpark-BOM-IoT-Button.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\smartmasjid-hardware\Design Files\IoT-Button-v1.2\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\smartmasjid-hardware\Design Files\IoT-Button-v1.2\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="2 Boards" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="500 Boards" sheetId="4" r:id="rId4"/>
     <sheet name="3000 Boards" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
@@ -712,7 +712,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
@@ -1446,6 +1446,33 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="25" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="25" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
@@ -1477,33 +1504,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="25" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="25" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1549,7 +1549,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1598,7 +1598,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1652,7 +1652,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1706,7 +1706,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1760,7 +1760,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1814,7 +1814,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2146,15 +2146,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="92"/>
-      <c r="L1" s="92"/>
-      <c r="M1" s="92"/>
-      <c r="N1" s="92"/>
-      <c r="O1" s="92"/>
-      <c r="P1" s="92"/>
-      <c r="Q1" s="92"/>
-      <c r="R1" s="92"/>
-      <c r="S1" s="93"/>
+      <c r="K1" s="101"/>
+      <c r="L1" s="101"/>
+      <c r="M1" s="101"/>
+      <c r="N1" s="101"/>
+      <c r="O1" s="101"/>
+      <c r="P1" s="101"/>
+      <c r="Q1" s="101"/>
+      <c r="R1" s="101"/>
+      <c r="S1" s="102"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2204,7 +2204,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="94"/>
+      <c r="S3" s="103"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2229,7 +2229,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="95"/>
+      <c r="S4" s="104"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2254,7 +2254,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="95"/>
+      <c r="S5" s="104"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2275,7 +2275,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="95"/>
+      <c r="S6" s="104"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2296,7 +2296,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="95"/>
+      <c r="S7" s="104"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2317,7 +2317,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="95"/>
+      <c r="S8" s="104"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -3170,13 +3170,13 @@
       <c r="D24" s="37" t="s">
         <v>219</v>
       </c>
-      <c r="E24" s="96" t="s">
+      <c r="E24" s="86" t="s">
         <v>220</v>
       </c>
       <c r="F24" s="37" t="s">
         <v>221</v>
       </c>
-      <c r="G24" s="96" t="s">
+      <c r="G24" s="86" t="s">
         <v>222</v>
       </c>
       <c r="H24" s="37" t="s">
@@ -3612,53 +3612,53 @@
         <f t="shared" ref="B32" si="11">ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="97" t="s">
+      <c r="C32" s="87" t="s">
         <v>18</v>
       </c>
-      <c r="D32" s="98" t="s">
+      <c r="D32" s="88" t="s">
         <v>182</v>
       </c>
-      <c r="E32" s="98" t="s">
+      <c r="E32" s="88" t="s">
         <v>51</v>
       </c>
-      <c r="F32" s="98" t="s">
+      <c r="F32" s="88" t="s">
         <v>65</v>
       </c>
-      <c r="G32" s="98" t="s">
+      <c r="G32" s="88" t="s">
         <v>81</v>
       </c>
-      <c r="H32" s="98" t="s">
+      <c r="H32" s="88" t="s">
         <v>86</v>
       </c>
-      <c r="I32" s="98" t="s">
-        <v>134</v>
-      </c>
-      <c r="J32" s="98" t="s">
+      <c r="I32" s="88" t="s">
+        <v>134</v>
+      </c>
+      <c r="J32" s="88" t="s">
         <v>112</v>
       </c>
-      <c r="K32" s="98" t="s">
+      <c r="K32" s="88" t="s">
         <v>183</v>
       </c>
-      <c r="L32" s="98">
-        <v>1</v>
-      </c>
-      <c r="M32" s="99">
+      <c r="L32" s="88">
+        <v>1</v>
+      </c>
+      <c r="M32" s="89">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="N32" s="99">
+      <c r="N32" s="89">
         <v>100</v>
       </c>
-      <c r="O32" s="100" t="s">
-        <v>136</v>
-      </c>
-      <c r="P32" s="101" t="s">
-        <v>134</v>
-      </c>
-      <c r="Q32" s="101" t="s">
-        <v>134</v>
-      </c>
-      <c r="R32" s="102" t="s">
+      <c r="O32" s="90" t="s">
+        <v>136</v>
+      </c>
+      <c r="P32" s="91" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q32" s="91" t="s">
+        <v>134</v>
+      </c>
+      <c r="R32" s="92" t="s">
         <v>183</v>
       </c>
       <c r="S32" s="55"/>
@@ -4121,17 +4121,17 @@
       <c r="K41" s="45"/>
       <c r="L41" s="45"/>
       <c r="M41" s="45"/>
-      <c r="N41" s="86" t="s">
+      <c r="N41" s="95" t="s">
         <v>5</v>
       </c>
-      <c r="O41" s="87"/>
-      <c r="P41" s="87"/>
+      <c r="O41" s="96"/>
+      <c r="P41" s="96"/>
       <c r="Q41" s="47">
-        <f>SUM(Q11:Q40)</f>
-        <v>32.793300000000009</v>
-      </c>
-      <c r="R41" s="88"/>
-      <c r="S41" s="89"/>
+        <f>SUM(Q10:Q40)</f>
+        <v>32.973300000000002</v>
+      </c>
+      <c r="R41" s="97"/>
+      <c r="S41" s="98"/>
     </row>
     <row r="42" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="56"/>
@@ -4147,17 +4147,17 @@
       <c r="K42" s="10"/>
       <c r="L42" s="10"/>
       <c r="M42" s="10"/>
-      <c r="N42" s="86" t="s">
+      <c r="N42" s="95" t="s">
         <v>6</v>
       </c>
-      <c r="O42" s="87"/>
-      <c r="P42" s="87"/>
+      <c r="O42" s="96"/>
+      <c r="P42" s="96"/>
       <c r="Q42" s="48">
         <f>Q41/2</f>
-        <v>16.396650000000005</v>
-      </c>
-      <c r="R42" s="90"/>
-      <c r="S42" s="91"/>
+        <v>16.486650000000001</v>
+      </c>
+      <c r="R42" s="99"/>
+      <c r="S42" s="100"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -4241,15 +4241,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="92"/>
-      <c r="L1" s="92"/>
-      <c r="M1" s="92"/>
-      <c r="N1" s="92"/>
-      <c r="O1" s="92"/>
-      <c r="P1" s="92"/>
-      <c r="Q1" s="92"/>
-      <c r="R1" s="92"/>
-      <c r="S1" s="93"/>
+      <c r="K1" s="101"/>
+      <c r="L1" s="101"/>
+      <c r="M1" s="101"/>
+      <c r="N1" s="101"/>
+      <c r="O1" s="101"/>
+      <c r="P1" s="101"/>
+      <c r="Q1" s="101"/>
+      <c r="R1" s="101"/>
+      <c r="S1" s="102"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -4299,7 +4299,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="94"/>
+      <c r="S3" s="103"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -4324,7 +4324,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="95"/>
+      <c r="S4" s="104"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -4349,7 +4349,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="95"/>
+      <c r="S5" s="104"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -4370,7 +4370,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="95"/>
+      <c r="S6" s="104"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -4391,7 +4391,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="95"/>
+      <c r="S7" s="104"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -4412,7 +4412,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="95"/>
+      <c r="S8" s="104"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -5265,13 +5265,13 @@
       <c r="D24" s="37" t="s">
         <v>219</v>
       </c>
-      <c r="E24" s="96" t="s">
+      <c r="E24" s="86" t="s">
         <v>220</v>
       </c>
       <c r="F24" s="37" t="s">
         <v>221</v>
       </c>
-      <c r="G24" s="96" t="s">
+      <c r="G24" s="86" t="s">
         <v>222</v>
       </c>
       <c r="H24" s="37" t="s">
@@ -5707,56 +5707,56 @@
         <f t="shared" ref="B32" si="11">ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="97" t="s">
+      <c r="C32" s="87" t="s">
         <v>18</v>
       </c>
-      <c r="D32" s="98" t="s">
+      <c r="D32" s="88" t="s">
         <v>182</v>
       </c>
-      <c r="E32" s="98" t="s">
+      <c r="E32" s="88" t="s">
         <v>51</v>
       </c>
-      <c r="F32" s="98" t="s">
+      <c r="F32" s="88" t="s">
         <v>65</v>
       </c>
-      <c r="G32" s="98" t="s">
+      <c r="G32" s="88" t="s">
         <v>81</v>
       </c>
-      <c r="H32" s="98" t="s">
+      <c r="H32" s="88" t="s">
         <v>86</v>
       </c>
-      <c r="I32" s="98" t="s">
-        <v>134</v>
-      </c>
-      <c r="J32" s="98" t="s">
+      <c r="I32" s="88" t="s">
+        <v>134</v>
+      </c>
+      <c r="J32" s="88" t="s">
         <v>112</v>
       </c>
-      <c r="K32" s="98" t="s">
+      <c r="K32" s="88" t="s">
         <v>183</v>
       </c>
-      <c r="L32" s="98">
-        <v>1</v>
-      </c>
-      <c r="M32" s="98">
+      <c r="L32" s="88">
+        <v>1</v>
+      </c>
+      <c r="M32" s="88">
         <f t="shared" ref="M32" si="12">L32*5</f>
         <v>5</v>
       </c>
-      <c r="N32" s="99" t="s">
-        <v>134</v>
-      </c>
-      <c r="O32" s="100" t="s">
-        <v>136</v>
-      </c>
-      <c r="P32" s="101" t="s">
-        <v>134</v>
-      </c>
-      <c r="Q32" s="103" t="s">
-        <v>134</v>
-      </c>
-      <c r="R32" s="102" t="s">
+      <c r="N32" s="89" t="s">
+        <v>134</v>
+      </c>
+      <c r="O32" s="90" t="s">
+        <v>136</v>
+      </c>
+      <c r="P32" s="91" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q32" s="93" t="s">
+        <v>134</v>
+      </c>
+      <c r="R32" s="92" t="s">
         <v>183</v>
       </c>
-      <c r="S32" s="104"/>
+      <c r="S32" s="94"/>
     </row>
     <row r="33" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A33" s="1"/>
@@ -6216,17 +6216,17 @@
       <c r="K41" s="45"/>
       <c r="L41" s="45"/>
       <c r="M41" s="45"/>
-      <c r="N41" s="86" t="s">
+      <c r="N41" s="95" t="s">
         <v>5</v>
       </c>
-      <c r="O41" s="87"/>
-      <c r="P41" s="87"/>
+      <c r="O41" s="96"/>
+      <c r="P41" s="96"/>
       <c r="Q41" s="47">
-        <f>SUM(Q11:Q40)</f>
-        <v>63.825400000000002</v>
-      </c>
-      <c r="R41" s="88"/>
-      <c r="S41" s="89"/>
+        <f>SUM(Q10:Q40)</f>
+        <v>64.005400000000009</v>
+      </c>
+      <c r="R41" s="97"/>
+      <c r="S41" s="98"/>
     </row>
     <row r="42" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
@@ -6242,17 +6242,17 @@
       <c r="K42" s="10"/>
       <c r="L42" s="10"/>
       <c r="M42" s="10"/>
-      <c r="N42" s="86" t="s">
+      <c r="N42" s="95" t="s">
         <v>6</v>
       </c>
-      <c r="O42" s="87"/>
-      <c r="P42" s="87"/>
+      <c r="O42" s="96"/>
+      <c r="P42" s="96"/>
       <c r="Q42" s="48">
         <f>Q41/5</f>
-        <v>12.765080000000001</v>
-      </c>
-      <c r="R42" s="90"/>
-      <c r="S42" s="91"/>
+        <v>12.801080000000002</v>
+      </c>
+      <c r="R42" s="99"/>
+      <c r="S42" s="100"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -6336,15 +6336,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="92"/>
-      <c r="L1" s="92"/>
-      <c r="M1" s="92"/>
-      <c r="N1" s="92"/>
-      <c r="O1" s="92"/>
-      <c r="P1" s="92"/>
-      <c r="Q1" s="92"/>
-      <c r="R1" s="92"/>
-      <c r="S1" s="93"/>
+      <c r="K1" s="101"/>
+      <c r="L1" s="101"/>
+      <c r="M1" s="101"/>
+      <c r="N1" s="101"/>
+      <c r="O1" s="101"/>
+      <c r="P1" s="101"/>
+      <c r="Q1" s="101"/>
+      <c r="R1" s="101"/>
+      <c r="S1" s="102"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -6394,7 +6394,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="94"/>
+      <c r="S3" s="103"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -6419,7 +6419,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="95"/>
+      <c r="S4" s="104"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -6444,7 +6444,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="95"/>
+      <c r="S5" s="104"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -6465,7 +6465,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="95"/>
+      <c r="S6" s="104"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -6486,7 +6486,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="95"/>
+      <c r="S7" s="104"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -6507,7 +6507,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="95"/>
+      <c r="S8" s="104"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -7360,13 +7360,13 @@
       <c r="D24" s="37" t="s">
         <v>219</v>
       </c>
-      <c r="E24" s="96" t="s">
+      <c r="E24" s="86" t="s">
         <v>220</v>
       </c>
       <c r="F24" s="37" t="s">
         <v>221</v>
       </c>
-      <c r="G24" s="96" t="s">
+      <c r="G24" s="86" t="s">
         <v>222</v>
       </c>
       <c r="H24" s="37" t="s">
@@ -7799,58 +7799,58 @@
         <f t="shared" ref="B32" si="8">ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="97" t="s">
+      <c r="C32" s="87" t="s">
         <v>18</v>
       </c>
-      <c r="D32" s="98" t="s">
+      <c r="D32" s="88" t="s">
         <v>182</v>
       </c>
-      <c r="E32" s="98" t="s">
+      <c r="E32" s="88" t="s">
         <v>51</v>
       </c>
-      <c r="F32" s="98" t="s">
+      <c r="F32" s="88" t="s">
         <v>65</v>
       </c>
-      <c r="G32" s="98" t="s">
+      <c r="G32" s="88" t="s">
         <v>81</v>
       </c>
-      <c r="H32" s="98" t="s">
+      <c r="H32" s="88" t="s">
         <v>86</v>
       </c>
-      <c r="I32" s="98" t="s">
-        <v>134</v>
-      </c>
-      <c r="J32" s="98" t="s">
+      <c r="I32" s="88" t="s">
+        <v>134</v>
+      </c>
+      <c r="J32" s="88" t="s">
         <v>112</v>
       </c>
-      <c r="K32" s="98" t="s">
+      <c r="K32" s="88" t="s">
         <v>183</v>
       </c>
-      <c r="L32" s="98">
-        <v>1</v>
-      </c>
-      <c r="M32" s="99">
+      <c r="L32" s="88">
+        <v>1</v>
+      </c>
+      <c r="M32" s="89">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="N32" s="99" t="s">
-        <v>134</v>
-      </c>
-      <c r="O32" s="100" t="s">
-        <v>136</v>
-      </c>
-      <c r="P32" s="101" t="s">
-        <v>134</v>
-      </c>
-      <c r="Q32" s="103" t="s">
-        <v>134</v>
-      </c>
-      <c r="R32" s="102" t="s">
+      <c r="N32" s="89" t="s">
+        <v>134</v>
+      </c>
+      <c r="O32" s="90" t="s">
+        <v>136</v>
+      </c>
+      <c r="P32" s="91" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q32" s="93" t="s">
+        <v>134</v>
+      </c>
+      <c r="R32" s="92" t="s">
         <v>183</v>
       </c>
-      <c r="S32" s="104"/>
-    </row>
-    <row r="33" spans="1:19" s="58" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="S32" s="94"/>
+    </row>
+    <row r="33" spans="1:19" s="58" customFormat="1" ht="24" x14ac:dyDescent="0.25">
       <c r="A33" s="56"/>
       <c r="B33" s="46">
         <f>ROW(B33) - ROW($B$9)</f>
@@ -8308,17 +8308,17 @@
       <c r="K41" s="45"/>
       <c r="L41" s="45"/>
       <c r="M41" s="45"/>
-      <c r="N41" s="86" t="s">
+      <c r="N41" s="95" t="s">
         <v>5</v>
       </c>
-      <c r="O41" s="87"/>
-      <c r="P41" s="87"/>
+      <c r="O41" s="96"/>
+      <c r="P41" s="96"/>
       <c r="Q41" s="47">
-        <f>SUM(Q11:Q40)</f>
-        <v>513.7921</v>
-      </c>
-      <c r="R41" s="88"/>
-      <c r="S41" s="89"/>
+        <f>SUM(Q10:Q40)</f>
+        <v>515.23210000000006</v>
+      </c>
+      <c r="R41" s="97"/>
+      <c r="S41" s="98"/>
     </row>
     <row r="42" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
@@ -8334,17 +8334,17 @@
       <c r="K42" s="10"/>
       <c r="L42" s="10"/>
       <c r="M42" s="10"/>
-      <c r="N42" s="86" t="s">
+      <c r="N42" s="95" t="s">
         <v>6</v>
       </c>
-      <c r="O42" s="87"/>
-      <c r="P42" s="87"/>
+      <c r="O42" s="96"/>
+      <c r="P42" s="96"/>
       <c r="Q42" s="48">
         <f>Q41/50</f>
-        <v>10.275842000000001</v>
-      </c>
-      <c r="R42" s="90"/>
-      <c r="S42" s="91"/>
+        <v>10.304642000000001</v>
+      </c>
+      <c r="R42" s="99"/>
+      <c r="S42" s="100"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -8428,15 +8428,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="92"/>
-      <c r="L1" s="92"/>
-      <c r="M1" s="92"/>
-      <c r="N1" s="92"/>
-      <c r="O1" s="92"/>
-      <c r="P1" s="92"/>
-      <c r="Q1" s="92"/>
-      <c r="R1" s="92"/>
-      <c r="S1" s="93"/>
+      <c r="K1" s="101"/>
+      <c r="L1" s="101"/>
+      <c r="M1" s="101"/>
+      <c r="N1" s="101"/>
+      <c r="O1" s="101"/>
+      <c r="P1" s="101"/>
+      <c r="Q1" s="101"/>
+      <c r="R1" s="101"/>
+      <c r="S1" s="102"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -8486,7 +8486,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="94"/>
+      <c r="S3" s="103"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -8511,7 +8511,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="95"/>
+      <c r="S4" s="104"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -8536,7 +8536,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="95"/>
+      <c r="S5" s="104"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -8557,7 +8557,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="95"/>
+      <c r="S6" s="104"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -8578,7 +8578,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="95"/>
+      <c r="S7" s="104"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -8599,7 +8599,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="95"/>
+      <c r="S8" s="104"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -10343,17 +10343,17 @@
       <c r="K40" s="45"/>
       <c r="L40" s="45"/>
       <c r="M40" s="45"/>
-      <c r="N40" s="86" t="s">
+      <c r="N40" s="95" t="s">
         <v>5</v>
       </c>
-      <c r="O40" s="87"/>
-      <c r="P40" s="87"/>
+      <c r="O40" s="96"/>
+      <c r="P40" s="96"/>
       <c r="Q40" s="47">
-        <f>SUM(Q11:Q39)</f>
-        <v>179.83190000000005</v>
-      </c>
-      <c r="R40" s="88"/>
-      <c r="S40" s="89"/>
+        <f>SUM(Q10:Q39)</f>
+        <v>189.71190000000004</v>
+      </c>
+      <c r="R40" s="97"/>
+      <c r="S40" s="98"/>
     </row>
     <row r="41" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
@@ -10369,17 +10369,17 @@
       <c r="K41" s="10"/>
       <c r="L41" s="10"/>
       <c r="M41" s="10"/>
-      <c r="N41" s="86" t="s">
+      <c r="N41" s="95" t="s">
         <v>6</v>
       </c>
-      <c r="O41" s="87"/>
-      <c r="P41" s="87"/>
+      <c r="O41" s="96"/>
+      <c r="P41" s="96"/>
       <c r="Q41" s="48">
         <f>Q40/500</f>
-        <v>0.35966380000000009</v>
-      </c>
-      <c r="R41" s="90"/>
-      <c r="S41" s="91"/>
+        <v>0.37942380000000009</v>
+      </c>
+      <c r="R41" s="99"/>
+      <c r="S41" s="100"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -10462,15 +10462,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="92"/>
-      <c r="L1" s="92"/>
-      <c r="M1" s="92"/>
-      <c r="N1" s="92"/>
-      <c r="O1" s="92"/>
-      <c r="P1" s="92"/>
-      <c r="Q1" s="92"/>
-      <c r="R1" s="92"/>
-      <c r="S1" s="93"/>
+      <c r="K1" s="101"/>
+      <c r="L1" s="101"/>
+      <c r="M1" s="101"/>
+      <c r="N1" s="101"/>
+      <c r="O1" s="101"/>
+      <c r="P1" s="101"/>
+      <c r="Q1" s="101"/>
+      <c r="R1" s="101"/>
+      <c r="S1" s="102"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -10520,7 +10520,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="94"/>
+      <c r="S3" s="103"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -10545,7 +10545,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="95"/>
+      <c r="S4" s="104"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -10570,7 +10570,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="95"/>
+      <c r="S5" s="104"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -10591,7 +10591,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="95"/>
+      <c r="S6" s="104"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -10612,7 +10612,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="95"/>
+      <c r="S7" s="104"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -10633,7 +10633,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="95"/>
+      <c r="S8" s="104"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -12377,17 +12377,17 @@
       <c r="K40" s="45"/>
       <c r="L40" s="45"/>
       <c r="M40" s="45"/>
-      <c r="N40" s="86" t="s">
+      <c r="N40" s="95" t="s">
         <v>5</v>
       </c>
-      <c r="O40" s="87"/>
-      <c r="P40" s="87"/>
+      <c r="O40" s="96"/>
+      <c r="P40" s="96"/>
       <c r="Q40" s="47">
-        <f>SUM(Q11:Q39)</f>
-        <v>175.00190000000006</v>
-      </c>
-      <c r="R40" s="88"/>
-      <c r="S40" s="89"/>
+        <f>SUM(Q10:Q39)</f>
+        <v>184.88190000000006</v>
+      </c>
+      <c r="R40" s="97"/>
+      <c r="S40" s="98"/>
     </row>
     <row r="41" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
@@ -12403,17 +12403,17 @@
       <c r="K41" s="10"/>
       <c r="L41" s="10"/>
       <c r="M41" s="10"/>
-      <c r="N41" s="86" t="s">
+      <c r="N41" s="95" t="s">
         <v>6</v>
       </c>
-      <c r="O41" s="87"/>
-      <c r="P41" s="87"/>
+      <c r="O41" s="96"/>
+      <c r="P41" s="96"/>
       <c r="Q41" s="48">
         <f>Q40/500</f>
-        <v>0.35000380000000014</v>
-      </c>
-      <c r="R41" s="90"/>
-      <c r="S41" s="91"/>
+        <v>0.36976380000000014</v>
+      </c>
+      <c r="R41" s="99"/>
+      <c r="S41" s="100"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
#23 R15 added in eSpark BOM Quantity 2.5 and 50 Boards.
</commit_message>
<xml_diff>
--- a/Design Files/IoT-Button-v1.2/BOM/eSpark-BOM-IoT-Button.xlsx
+++ b/Design Files/IoT-Button-v1.2/BOM/eSpark-BOM-IoT-Button.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\smartmasjid-hardware\Design Files\IoT-Button-v1.2\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\smartmasjid-hardware\Design Files\IoT-Button-v1.2\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="2 Boards" sheetId="1" r:id="rId1"/>
@@ -18,12 +18,12 @@
     <sheet name="500 Boards" sheetId="4" r:id="rId4"/>
     <sheet name="3000 Boards" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1670" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1700" uniqueCount="233">
   <si>
     <t>Component list</t>
   </si>
@@ -707,12 +707,27 @@
   </si>
   <si>
     <t>C5310968</t>
+  </si>
+  <si>
+    <t>R15</t>
+  </si>
+  <si>
+    <t>RES SMD 1K OHM 1% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>RC0603FR-071KL</t>
+  </si>
+  <si>
+    <t>C22548</t>
+  </si>
+  <si>
+    <t>1K</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
@@ -1549,7 +1564,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1598,7 +1613,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1652,7 +1667,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1706,7 +1721,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1760,7 +1775,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1814,7 +1829,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2112,7 +2127,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S42"/>
+  <dimension ref="A1:S43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="26" customWidth="1"/>
@@ -2435,7 +2450,7 @@
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="56"/>
       <c r="B11" s="46">
-        <f>ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B41" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="67" t="s">
@@ -2482,7 +2497,7 @@
         <v>5.1999999999999998E-3</v>
       </c>
       <c r="Q11" s="50">
-        <f t="shared" ref="Q11" si="0">P11*N11</f>
+        <f t="shared" ref="Q11" si="1">P11*N11</f>
         <v>0.52</v>
       </c>
       <c r="R11" s="49"/>
@@ -2491,7 +2506,7 @@
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="56"/>
       <c r="B12" s="46">
-        <f t="shared" ref="B12:B40" si="1">ROW(B12) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C12" s="67" t="s">
@@ -2547,7 +2562,7 @@
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="56"/>
       <c r="B13" s="46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C13" s="67" t="s">
@@ -2581,7 +2596,7 @@
         <v>1</v>
       </c>
       <c r="M13" s="37">
-        <f t="shared" ref="M13:M40" si="2">L13*2</f>
+        <f t="shared" ref="M13:M41" si="2">L13*2</f>
         <v>2</v>
       </c>
       <c r="N13" s="49">
@@ -2602,8 +2617,8 @@
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="56"/>
-      <c r="B14" s="72">
-        <f t="shared" si="1"/>
+      <c r="B14" s="46">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C14" s="67" t="s">
@@ -2659,7 +2674,7 @@
     <row r="15" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A15" s="56"/>
       <c r="B15" s="46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C15" s="67" t="s">
@@ -2713,7 +2728,7 @@
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="56"/>
       <c r="B16" s="46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C16" s="68" t="s">
@@ -2769,7 +2784,7 @@
     <row r="17" spans="1:19" ht="36" x14ac:dyDescent="0.25">
       <c r="A17" s="56"/>
       <c r="B17" s="46">
-        <f>ROW(B17) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C17" s="67" t="s">
@@ -2825,7 +2840,7 @@
     <row r="18" spans="1:19" ht="48" x14ac:dyDescent="0.25">
       <c r="A18" s="56"/>
       <c r="B18" s="46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C18" s="68" t="s">
@@ -2881,7 +2896,7 @@
     <row r="19" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A19" s="56"/>
       <c r="B19" s="46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C19" s="67" t="s">
@@ -2937,7 +2952,7 @@
     <row r="20" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A20" s="56"/>
       <c r="B20" s="46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C20" s="67" t="s">
@@ -2993,7 +3008,7 @@
     <row r="21" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A21" s="56"/>
       <c r="B21" s="46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C21" s="68" t="s">
@@ -3049,7 +3064,7 @@
     <row r="22" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A22" s="56"/>
       <c r="B22" s="46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C22" s="67" t="s">
@@ -3105,7 +3120,7 @@
     <row r="23" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A23" s="56"/>
       <c r="B23" s="46">
-        <f>ROW(B23) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C23" s="67" t="s">
@@ -3161,7 +3176,7 @@
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="56"/>
       <c r="B24" s="46">
-        <f>ROW(B24) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C24" s="67" t="s">
@@ -3214,10 +3229,10 @@
       <c r="R24" s="37"/>
       <c r="S24" s="55"/>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A25" s="56"/>
-      <c r="B25" s="73">
-        <f t="shared" si="1"/>
+      <c r="B25" s="46">
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C25" s="74" t="s">
@@ -3226,7 +3241,7 @@
       <c r="D25" s="75" t="s">
         <v>208</v>
       </c>
-      <c r="E25" s="75" t="s">
+      <c r="E25" s="49" t="s">
         <v>172</v>
       </c>
       <c r="F25" s="75" t="s">
@@ -3273,7 +3288,7 @@
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="56"/>
       <c r="B26" s="46">
-        <f>ROW(B26) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C26" s="68" t="s">
@@ -3329,7 +3344,7 @@
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="56"/>
       <c r="B27" s="46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C27" s="68" t="s">
@@ -3385,7 +3400,7 @@
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="56"/>
       <c r="B28" s="46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C28" s="67" t="s">
@@ -3441,7 +3456,7 @@
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="56"/>
       <c r="B29" s="46">
-        <f>ROW(B29) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C29" s="67" t="s">
@@ -3497,7 +3512,7 @@
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="56"/>
       <c r="B30" s="46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C30" s="68" t="s">
@@ -3553,7 +3568,7 @@
     <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31" s="56"/>
       <c r="B31" s="46">
-        <f>ROW(B31) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C31" s="68" t="s">
@@ -3608,8 +3623,8 @@
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A32" s="56"/>
-      <c r="B32" s="72">
-        <f t="shared" ref="B32" si="11">ROW(B32) - ROW($B$9)</f>
+      <c r="B32" s="46">
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C32" s="87" t="s">
@@ -3663,38 +3678,38 @@
       </c>
       <c r="S32" s="55"/>
     </row>
-    <row r="33" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33" s="56"/>
       <c r="B33" s="46">
-        <f>ROW(B33) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C33" s="68" t="s">
-        <v>187</v>
-      </c>
-      <c r="D33" s="37" t="s">
-        <v>33</v>
-      </c>
-      <c r="E33" s="37" t="s">
-        <v>185</v>
-      </c>
-      <c r="F33" s="37" t="s">
-        <v>135</v>
-      </c>
-      <c r="G33" s="37" t="s">
-        <v>186</v>
-      </c>
-      <c r="H33" s="37" t="s">
-        <v>184</v>
+      <c r="C33" s="67" t="s">
+        <v>18</v>
+      </c>
+      <c r="D33" s="49" t="s">
+        <v>228</v>
+      </c>
+      <c r="E33" s="85" t="s">
+        <v>229</v>
+      </c>
+      <c r="F33" s="49" t="s">
+        <v>65</v>
+      </c>
+      <c r="G33" s="85" t="s">
+        <v>230</v>
+      </c>
+      <c r="H33" s="49" t="s">
+        <v>86</v>
       </c>
       <c r="I33" s="37" t="s">
         <v>134</v>
       </c>
       <c r="J33" s="37" t="s">
-        <v>197</v>
+        <v>231</v>
       </c>
       <c r="K33" s="37" t="s">
-        <v>134</v>
+        <v>232</v>
       </c>
       <c r="L33" s="37">
         <v>1</v>
@@ -3703,219 +3718,219 @@
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="N33" s="49">
-        <v>5</v>
+      <c r="N33" s="37">
+        <v>100</v>
       </c>
       <c r="O33" s="59" t="s">
         <v>136</v>
       </c>
       <c r="P33" s="38">
-        <v>0.1336</v>
+        <v>1E-3</v>
       </c>
       <c r="Q33" s="50">
-        <f t="shared" ref="Q33" si="12">P33*N33</f>
-        <v>0.66799999999999993</v>
-      </c>
-      <c r="R33" s="49"/>
+        <f>P33*N33</f>
+        <v>0.1</v>
+      </c>
+      <c r="R33" s="76"/>
       <c r="S33" s="55"/>
     </row>
-    <row r="34" spans="1:19" ht="36" x14ac:dyDescent="0.25">
-      <c r="A34" s="61"/>
-      <c r="B34" s="72">
-        <f t="shared" ref="B34" si="13">ROW(B34) - ROW($B$9)</f>
+    <row r="34" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+      <c r="A34" s="56"/>
+      <c r="B34" s="46">
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="C34" s="68" t="s">
         <v>187</v>
       </c>
-      <c r="D34" s="49" t="s">
-        <v>188</v>
-      </c>
-      <c r="E34" s="49" t="s">
-        <v>189</v>
-      </c>
-      <c r="F34" s="49" t="s">
+      <c r="D34" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="E34" s="37" t="s">
+        <v>185</v>
+      </c>
+      <c r="F34" s="37" t="s">
         <v>135</v>
       </c>
-      <c r="G34" s="49" t="s">
-        <v>190</v>
-      </c>
-      <c r="H34" s="49" t="s">
-        <v>191</v>
-      </c>
-      <c r="I34" s="49" t="s">
-        <v>134</v>
-      </c>
-      <c r="J34" s="49" t="s">
-        <v>192</v>
-      </c>
-      <c r="K34" s="49" t="s">
-        <v>134</v>
-      </c>
-      <c r="L34" s="49">
-        <v>2</v>
+      <c r="G34" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="H34" s="37" t="s">
+        <v>184</v>
+      </c>
+      <c r="I34" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="J34" s="37" t="s">
+        <v>197</v>
+      </c>
+      <c r="K34" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="L34" s="37">
+        <v>1</v>
       </c>
       <c r="M34" s="37">
         <f t="shared" si="2"/>
-        <v>4</v>
-      </c>
-      <c r="N34" s="62">
-        <v>10</v>
-      </c>
-      <c r="O34" s="60" t="s">
-        <v>136</v>
-      </c>
-      <c r="P34" s="50">
-        <v>4.8300000000000003E-2</v>
-      </c>
-      <c r="Q34" s="63">
-        <f>P34*N34</f>
-        <v>0.48300000000000004</v>
-      </c>
-      <c r="R34" s="62"/>
-      <c r="S34" s="64"/>
+        <v>2</v>
+      </c>
+      <c r="N34" s="49">
+        <v>5</v>
+      </c>
+      <c r="O34" s="59" t="s">
+        <v>136</v>
+      </c>
+      <c r="P34" s="38">
+        <v>0.1336</v>
+      </c>
+      <c r="Q34" s="50">
+        <f t="shared" ref="Q34" si="11">P34*N34</f>
+        <v>0.66799999999999993</v>
+      </c>
+      <c r="R34" s="49"/>
+      <c r="S34" s="55"/>
     </row>
     <row r="35" spans="1:19" ht="36" x14ac:dyDescent="0.25">
-      <c r="A35" s="56"/>
+      <c r="A35" s="61"/>
       <c r="B35" s="46">
-        <f>ROW(B35) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C35" s="67" t="s">
+      <c r="C35" s="68" t="s">
         <v>187</v>
       </c>
-      <c r="D35" s="37" t="s">
-        <v>193</v>
-      </c>
-      <c r="E35" s="37" t="s">
-        <v>194</v>
-      </c>
-      <c r="F35" s="37" t="s">
+      <c r="D35" s="49" t="s">
+        <v>188</v>
+      </c>
+      <c r="E35" s="49" t="s">
+        <v>189</v>
+      </c>
+      <c r="F35" s="49" t="s">
         <v>135</v>
       </c>
-      <c r="G35" s="37" t="s">
-        <v>195</v>
-      </c>
-      <c r="H35" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="I35" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="J35" s="37" t="s">
-        <v>196</v>
-      </c>
-      <c r="K35" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="L35" s="37">
-        <v>1</v>
+      <c r="G35" s="49" t="s">
+        <v>190</v>
+      </c>
+      <c r="H35" s="49" t="s">
+        <v>191</v>
+      </c>
+      <c r="I35" s="49" t="s">
+        <v>134</v>
+      </c>
+      <c r="J35" s="49" t="s">
+        <v>192</v>
+      </c>
+      <c r="K35" s="49" t="s">
+        <v>134</v>
+      </c>
+      <c r="L35" s="49">
+        <v>2</v>
       </c>
       <c r="M35" s="37">
         <f t="shared" si="2"/>
-        <v>2</v>
-      </c>
-      <c r="N35" s="49">
+        <v>4</v>
+      </c>
+      <c r="N35" s="62">
         <v>10</v>
       </c>
-      <c r="O35" s="59" t="s">
-        <v>136</v>
-      </c>
-      <c r="P35" s="38">
-        <v>6.4600000000000005E-2</v>
-      </c>
-      <c r="Q35" s="50">
-        <f t="shared" ref="Q35" si="14">P35*N35</f>
-        <v>0.64600000000000002</v>
-      </c>
-      <c r="R35" s="49"/>
-      <c r="S35" s="55"/>
-    </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="O35" s="60" t="s">
+        <v>136</v>
+      </c>
+      <c r="P35" s="50">
+        <v>4.8300000000000003E-2</v>
+      </c>
+      <c r="Q35" s="63">
+        <f>P35*N35</f>
+        <v>0.48300000000000004</v>
+      </c>
+      <c r="R35" s="62"/>
+      <c r="S35" s="64"/>
+    </row>
+    <row r="36" spans="1:19" ht="36" x14ac:dyDescent="0.25">
       <c r="A36" s="56"/>
       <c r="B36" s="46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="C36" s="68" t="s">
-        <v>17</v>
-      </c>
-      <c r="D36" s="49" t="s">
-        <v>34</v>
-      </c>
-      <c r="E36" s="49" t="s">
-        <v>53</v>
-      </c>
-      <c r="F36" s="49" t="s">
-        <v>66</v>
-      </c>
-      <c r="G36" s="49" t="s">
-        <v>83</v>
-      </c>
-      <c r="H36" s="49" t="s">
-        <v>96</v>
-      </c>
-      <c r="I36" s="49" t="s">
-        <v>134</v>
-      </c>
-      <c r="J36" s="49" t="s">
-        <v>114</v>
+      <c r="C36" s="67" t="s">
+        <v>187</v>
+      </c>
+      <c r="D36" s="37" t="s">
+        <v>193</v>
+      </c>
+      <c r="E36" s="37" t="s">
+        <v>194</v>
+      </c>
+      <c r="F36" s="37" t="s">
+        <v>135</v>
+      </c>
+      <c r="G36" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="H36" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="I36" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="J36" s="37" t="s">
+        <v>196</v>
       </c>
       <c r="K36" s="37" t="s">
         <v>134</v>
       </c>
-      <c r="L36" s="49">
+      <c r="L36" s="37">
         <v>1</v>
       </c>
       <c r="M36" s="37">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="N36" s="37">
-        <v>5</v>
-      </c>
-      <c r="O36" s="60" t="s">
-        <v>136</v>
-      </c>
-      <c r="P36" s="50">
-        <v>0.2079</v>
-      </c>
-      <c r="Q36" s="38">
-        <f>P36*N36</f>
-        <v>1.0395000000000001</v>
-      </c>
-      <c r="R36" s="37"/>
+      <c r="N36" s="49">
+        <v>10</v>
+      </c>
+      <c r="O36" s="59" t="s">
+        <v>136</v>
+      </c>
+      <c r="P36" s="38">
+        <v>6.4600000000000005E-2</v>
+      </c>
+      <c r="Q36" s="50">
+        <f t="shared" ref="Q36" si="12">P36*N36</f>
+        <v>0.64600000000000002</v>
+      </c>
+      <c r="R36" s="49"/>
       <c r="S36" s="55"/>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A37" s="56"/>
       <c r="B37" s="46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C37" s="68" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D37" s="49" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E37" s="49" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F37" s="49" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G37" s="49" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H37" s="49" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I37" s="49" t="s">
         <v>134</v>
       </c>
       <c r="J37" s="49" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K37" s="37" t="s">
         <v>134</v>
@@ -3927,109 +3942,111 @@
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="N37" s="49">
-        <v>3</v>
+      <c r="N37" s="37">
+        <v>5</v>
       </c>
       <c r="O37" s="60" t="s">
         <v>136</v>
       </c>
       <c r="P37" s="50">
-        <v>0.54569999999999996</v>
-      </c>
-      <c r="Q37" s="50">
-        <f t="shared" ref="Q37" si="15">P37*N37</f>
-        <v>1.6370999999999998</v>
-      </c>
-      <c r="R37" s="49"/>
+        <v>0.2079</v>
+      </c>
+      <c r="Q37" s="38">
+        <f>P37*N37</f>
+        <v>1.0395000000000001</v>
+      </c>
+      <c r="R37" s="37"/>
       <c r="S37" s="55"/>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="56"/>
       <c r="B38" s="46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C38" s="67" t="s">
-        <v>20</v>
-      </c>
-      <c r="D38" s="37" t="s">
-        <v>36</v>
-      </c>
-      <c r="E38" s="37" t="s">
-        <v>55</v>
-      </c>
-      <c r="F38" s="37" t="s">
-        <v>135</v>
-      </c>
-      <c r="G38" s="37" t="s">
-        <v>68</v>
-      </c>
-      <c r="H38" s="37" t="s">
-        <v>98</v>
-      </c>
-      <c r="I38" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="J38" s="37" t="s">
-        <v>116</v>
+      <c r="C38" s="68" t="s">
+        <v>19</v>
+      </c>
+      <c r="D38" s="49" t="s">
+        <v>35</v>
+      </c>
+      <c r="E38" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="F38" s="49" t="s">
+        <v>67</v>
+      </c>
+      <c r="G38" s="49" t="s">
+        <v>84</v>
+      </c>
+      <c r="H38" s="49" t="s">
+        <v>97</v>
+      </c>
+      <c r="I38" s="49" t="s">
+        <v>134</v>
+      </c>
+      <c r="J38" s="49" t="s">
+        <v>115</v>
       </c>
       <c r="K38" s="37" t="s">
         <v>134</v>
       </c>
-      <c r="L38" s="37">
+      <c r="L38" s="49">
         <v>1</v>
       </c>
       <c r="M38" s="37">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="N38" s="37">
+      <c r="N38" s="49">
         <v>3</v>
       </c>
-      <c r="O38" s="59" t="s">
-        <v>136</v>
-      </c>
-      <c r="P38" s="38">
-        <v>2.8589000000000002</v>
-      </c>
-      <c r="Q38" s="38">
-        <f>P38*N38</f>
-        <v>8.5767000000000007</v>
-      </c>
-      <c r="R38" s="37"/>
+      <c r="O38" s="60" t="s">
+        <v>136</v>
+      </c>
+      <c r="P38" s="50">
+        <v>0.54569999999999996</v>
+      </c>
+      <c r="Q38" s="50">
+        <f t="shared" ref="Q38" si="13">P38*N38</f>
+        <v>1.6370999999999998</v>
+      </c>
+      <c r="R38" s="49"/>
       <c r="S38" s="55"/>
     </row>
-    <row r="39" spans="1:19" ht="48" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A39" s="56"/>
       <c r="B39" s="46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C39" s="67" t="s">
-        <v>144</v>
+        <v>20</v>
       </c>
       <c r="D39" s="37" t="s">
-        <v>143</v>
+        <v>36</v>
       </c>
       <c r="E39" s="37" t="s">
-        <v>225</v>
+        <v>55</v>
       </c>
       <c r="F39" s="37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G39" s="37" t="s">
-        <v>134</v>
+        <v>68</v>
       </c>
       <c r="H39" s="37" t="s">
-        <v>134</v>
+        <v>98</v>
       </c>
       <c r="I39" s="37" t="s">
         <v>134</v>
       </c>
       <c r="J39" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="K39" s="37"/>
+        <v>116</v>
+      </c>
+      <c r="K39" s="37" t="s">
+        <v>134</v>
+      </c>
       <c r="L39" s="37">
         <v>1</v>
       </c>
@@ -4038,35 +4055,35 @@
         <v>2</v>
       </c>
       <c r="N39" s="37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O39" s="59" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="P39" s="38">
-        <v>4.67</v>
+        <v>2.8589000000000002</v>
       </c>
       <c r="Q39" s="38">
         <f>P39*N39</f>
-        <v>9.34</v>
+        <v>8.5767000000000007</v>
       </c>
       <c r="R39" s="37"/>
       <c r="S39" s="55"/>
     </row>
-    <row r="40" spans="1:19" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:19" ht="48" x14ac:dyDescent="0.25">
       <c r="A40" s="56"/>
       <c r="B40" s="46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="C40" s="67" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D40" s="37" t="s">
         <v>143</v>
       </c>
       <c r="E40" s="37" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F40" s="37" t="s">
         <v>134</v>
@@ -4091,79 +4108,133 @@
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="N40" s="49">
-        <v>1</v>
+      <c r="N40" s="37">
+        <v>2</v>
       </c>
       <c r="O40" s="59" t="s">
         <v>147</v>
       </c>
       <c r="P40" s="38">
+        <v>4.67</v>
+      </c>
+      <c r="Q40" s="38">
+        <f>P40*N40</f>
+        <v>9.34</v>
+      </c>
+      <c r="R40" s="37"/>
+      <c r="S40" s="55"/>
+    </row>
+    <row r="41" spans="1:19" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="56"/>
+      <c r="B41" s="46">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="C41" s="67" t="s">
+        <v>145</v>
+      </c>
+      <c r="D41" s="37" t="s">
+        <v>143</v>
+      </c>
+      <c r="E41" s="37" t="s">
+        <v>226</v>
+      </c>
+      <c r="F41" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="G41" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="H41" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="I41" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="J41" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="K41" s="37"/>
+      <c r="L41" s="37">
+        <v>1</v>
+      </c>
+      <c r="M41" s="37">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="N41" s="49">
+        <v>1</v>
+      </c>
+      <c r="O41" s="59" t="s">
+        <v>147</v>
+      </c>
+      <c r="P41" s="38">
         <v>0.35</v>
       </c>
-      <c r="Q40" s="50">
-        <f t="shared" ref="Q40" si="16">P40*N40</f>
+      <c r="Q41" s="50">
+        <f t="shared" ref="Q41" si="14">P41*N41</f>
         <v>0.35</v>
       </c>
-      <c r="R40" s="49"/>
-      <c r="S40" s="55"/>
-    </row>
-    <row r="41" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="56"/>
-      <c r="B41" s="40"/>
-      <c r="C41" s="41"/>
-      <c r="D41" s="42"/>
-      <c r="E41" s="43"/>
-      <c r="F41" s="44"/>
-      <c r="G41" s="45"/>
-      <c r="H41" s="44"/>
-      <c r="I41" s="45"/>
-      <c r="J41" s="44"/>
-      <c r="K41" s="45"/>
-      <c r="L41" s="45"/>
-      <c r="M41" s="45"/>
-      <c r="N41" s="95" t="s">
-        <v>5</v>
-      </c>
-      <c r="O41" s="96"/>
-      <c r="P41" s="96"/>
-      <c r="Q41" s="47">
-        <f>SUM(Q10:Q40)</f>
-        <v>32.973300000000002</v>
-      </c>
-      <c r="R41" s="97"/>
-      <c r="S41" s="98"/>
+      <c r="R41" s="49"/>
+      <c r="S41" s="55"/>
     </row>
     <row r="42" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="56"/>
-      <c r="B42" s="25"/>
-      <c r="C42" s="36"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="10"/>
-      <c r="F42" s="10"/>
-      <c r="G42" s="10"/>
-      <c r="H42" s="10"/>
-      <c r="I42" s="10"/>
-      <c r="J42" s="10"/>
-      <c r="K42" s="10"/>
-      <c r="L42" s="10"/>
-      <c r="M42" s="10"/>
+      <c r="B42" s="40"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="42"/>
+      <c r="E42" s="43"/>
+      <c r="F42" s="44"/>
+      <c r="G42" s="45"/>
+      <c r="H42" s="44"/>
+      <c r="I42" s="45"/>
+      <c r="J42" s="44"/>
+      <c r="K42" s="45"/>
+      <c r="L42" s="45"/>
+      <c r="M42" s="45"/>
       <c r="N42" s="95" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O42" s="96"/>
       <c r="P42" s="96"/>
-      <c r="Q42" s="48">
-        <f>Q41/2</f>
-        <v>16.486650000000001</v>
-      </c>
-      <c r="R42" s="99"/>
-      <c r="S42" s="100"/>
+      <c r="Q42" s="47">
+        <f>SUM(Q10:Q41)</f>
+        <v>33.073300000000003</v>
+      </c>
+      <c r="R42" s="97"/>
+      <c r="S42" s="98"/>
+    </row>
+    <row r="43" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="56"/>
+      <c r="B43" s="25"/>
+      <c r="C43" s="36"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="10"/>
+      <c r="M43" s="10"/>
+      <c r="N43" s="95" t="s">
+        <v>6</v>
+      </c>
+      <c r="O43" s="96"/>
+      <c r="P43" s="96"/>
+      <c r="Q43" s="48">
+        <f>Q42/2</f>
+        <v>16.536650000000002</v>
+      </c>
+      <c r="R43" s="99"/>
+      <c r="S43" s="100"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="N41:P41"/>
-    <mergeCell ref="R41:S42"/>
     <mergeCell ref="N42:P42"/>
+    <mergeCell ref="R42:S43"/>
+    <mergeCell ref="N43:P43"/>
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
   </mergeCells>
@@ -4182,33 +4253,34 @@
     <hyperlink ref="O30" r:id="rId12"/>
     <hyperlink ref="O26" r:id="rId13"/>
     <hyperlink ref="O31" r:id="rId14"/>
-    <hyperlink ref="O36" r:id="rId15"/>
-    <hyperlink ref="O37" r:id="rId16"/>
-    <hyperlink ref="O38" r:id="rId17"/>
+    <hyperlink ref="O37" r:id="rId15"/>
+    <hyperlink ref="O38" r:id="rId16"/>
+    <hyperlink ref="O39" r:id="rId17"/>
     <hyperlink ref="O10" r:id="rId18"/>
     <hyperlink ref="O14" r:id="rId19"/>
     <hyperlink ref="O23" r:id="rId20"/>
     <hyperlink ref="O25" r:id="rId21"/>
     <hyperlink ref="O29" r:id="rId22"/>
     <hyperlink ref="O32" r:id="rId23"/>
-    <hyperlink ref="O33" r:id="rId24"/>
-    <hyperlink ref="O34" r:id="rId25"/>
-    <hyperlink ref="O35" r:id="rId26"/>
+    <hyperlink ref="O34" r:id="rId24"/>
+    <hyperlink ref="O35" r:id="rId25"/>
+    <hyperlink ref="O36" r:id="rId26"/>
     <hyperlink ref="O17" r:id="rId27"/>
     <hyperlink ref="O28" r:id="rId28"/>
-    <hyperlink ref="O39" r:id="rId29"/>
-    <hyperlink ref="O40" r:id="rId30"/>
+    <hyperlink ref="O40" r:id="rId29"/>
+    <hyperlink ref="O41" r:id="rId30"/>
     <hyperlink ref="O24" r:id="rId31"/>
+    <hyperlink ref="O33" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId32"/>
-  <drawing r:id="rId33"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId33"/>
+  <drawing r:id="rId34"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S42"/>
+  <dimension ref="A1:S43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
@@ -4586,7 +4658,7 @@
     <row r="12" spans="1:19" s="58" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="56"/>
       <c r="B12" s="46">
-        <f t="shared" ref="B12:B40" si="0">ROW(B12) - ROW($B$9)</f>
+        <f t="shared" ref="B12:B41" si="0">ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
       <c r="C12" s="67" t="s">
@@ -5704,7 +5776,7 @@
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A32" s="1"/>
       <c r="B32" s="72">
-        <f t="shared" ref="B32" si="11">ROW(B32) - ROW($B$9)</f>
+        <f t="shared" ref="B32:B33" si="11">ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
       <c r="C32" s="87" t="s">
@@ -5758,38 +5830,38 @@
       </c>
       <c r="S32" s="94"/>
     </row>
-    <row r="33" spans="1:19" ht="24" x14ac:dyDescent="0.25">
-      <c r="A33" s="1"/>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A33" s="56"/>
       <c r="B33" s="46">
-        <f>ROW(B33) - ROW($B$9)</f>
+        <f t="shared" si="11"/>
         <v>24</v>
       </c>
-      <c r="C33" s="68" t="s">
-        <v>187</v>
-      </c>
-      <c r="D33" s="37" t="s">
-        <v>33</v>
-      </c>
-      <c r="E33" s="37" t="s">
-        <v>185</v>
-      </c>
-      <c r="F33" s="37" t="s">
-        <v>135</v>
-      </c>
-      <c r="G33" s="37" t="s">
-        <v>186</v>
-      </c>
-      <c r="H33" s="37" t="s">
-        <v>184</v>
+      <c r="C33" s="67" t="s">
+        <v>18</v>
+      </c>
+      <c r="D33" s="49" t="s">
+        <v>228</v>
+      </c>
+      <c r="E33" s="85" t="s">
+        <v>229</v>
+      </c>
+      <c r="F33" s="49" t="s">
+        <v>65</v>
+      </c>
+      <c r="G33" s="85" t="s">
+        <v>230</v>
+      </c>
+      <c r="H33" s="49" t="s">
+        <v>86</v>
       </c>
       <c r="I33" s="37" t="s">
         <v>134</v>
       </c>
       <c r="J33" s="37" t="s">
-        <v>197</v>
+        <v>231</v>
       </c>
       <c r="K33" s="37" t="s">
-        <v>134</v>
+        <v>232</v>
       </c>
       <c r="L33" s="37">
         <v>1</v>
@@ -5799,187 +5871,187 @@
         <v>5</v>
       </c>
       <c r="N33" s="37">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="O33" s="59" t="s">
         <v>136</v>
       </c>
       <c r="P33" s="38">
-        <v>0.1336</v>
-      </c>
-      <c r="Q33" s="38">
+        <v>1E-3</v>
+      </c>
+      <c r="Q33" s="50">
         <f>P33*N33</f>
-        <v>1.3359999999999999</v>
-      </c>
-      <c r="R33" s="37"/>
+        <v>0.1</v>
+      </c>
+      <c r="R33" s="76"/>
       <c r="S33" s="55"/>
     </row>
-    <row r="34" spans="1:19" ht="36" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
-      <c r="B34" s="72">
-        <f t="shared" ref="B34" si="13">ROW(B34) - ROW($B$9)</f>
+      <c r="B34" s="46">
+        <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
       <c r="C34" s="68" t="s">
         <v>187</v>
       </c>
-      <c r="D34" s="49" t="s">
-        <v>188</v>
-      </c>
-      <c r="E34" s="49" t="s">
-        <v>189</v>
-      </c>
-      <c r="F34" s="49" t="s">
+      <c r="D34" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="E34" s="37" t="s">
+        <v>185</v>
+      </c>
+      <c r="F34" s="37" t="s">
         <v>135</v>
       </c>
-      <c r="G34" s="49" t="s">
-        <v>190</v>
-      </c>
-      <c r="H34" s="49" t="s">
-        <v>191</v>
-      </c>
-      <c r="I34" s="49" t="s">
-        <v>134</v>
-      </c>
-      <c r="J34" s="49" t="s">
-        <v>192</v>
-      </c>
-      <c r="K34" s="49" t="s">
-        <v>134</v>
-      </c>
-      <c r="L34" s="49">
-        <v>2</v>
-      </c>
-      <c r="M34" s="49">
-        <f t="shared" ref="M34" si="14">L34*5</f>
+      <c r="G34" s="37" t="s">
+        <v>186</v>
+      </c>
+      <c r="H34" s="37" t="s">
+        <v>184</v>
+      </c>
+      <c r="I34" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="J34" s="37" t="s">
+        <v>197</v>
+      </c>
+      <c r="K34" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="L34" s="37">
+        <v>1</v>
+      </c>
+      <c r="M34" s="37">
+        <f>L34*5</f>
+        <v>5</v>
+      </c>
+      <c r="N34" s="37">
         <v>10</v>
       </c>
-      <c r="N34" s="49">
-        <v>20</v>
-      </c>
-      <c r="O34" s="60" t="s">
-        <v>136</v>
-      </c>
-      <c r="P34" s="50">
-        <v>4.8300000000000003E-2</v>
-      </c>
-      <c r="Q34" s="50">
-        <f t="shared" ref="Q34" si="15">P34*N34</f>
-        <v>0.96600000000000008</v>
-      </c>
-      <c r="R34" s="49"/>
+      <c r="O34" s="59" t="s">
+        <v>136</v>
+      </c>
+      <c r="P34" s="38">
+        <v>0.1336</v>
+      </c>
+      <c r="Q34" s="38">
+        <f>P34*N34</f>
+        <v>1.3359999999999999</v>
+      </c>
+      <c r="R34" s="37"/>
       <c r="S34" s="55"/>
     </row>
     <row r="35" spans="1:19" ht="36" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
-      <c r="B35" s="46">
-        <f>ROW(B35) - ROW($B$9)</f>
+      <c r="B35" s="72">
+        <f t="shared" ref="B35" si="13">ROW(B35) - ROW($B$9)</f>
         <v>26</v>
       </c>
-      <c r="C35" s="67" t="s">
+      <c r="C35" s="68" t="s">
         <v>187</v>
       </c>
-      <c r="D35" s="37" t="s">
+      <c r="D35" s="49" t="s">
+        <v>188</v>
+      </c>
+      <c r="E35" s="49" t="s">
+        <v>189</v>
+      </c>
+      <c r="F35" s="49" t="s">
+        <v>135</v>
+      </c>
+      <c r="G35" s="49" t="s">
+        <v>190</v>
+      </c>
+      <c r="H35" s="49" t="s">
+        <v>191</v>
+      </c>
+      <c r="I35" s="49" t="s">
+        <v>134</v>
+      </c>
+      <c r="J35" s="49" t="s">
+        <v>192</v>
+      </c>
+      <c r="K35" s="49" t="s">
+        <v>134</v>
+      </c>
+      <c r="L35" s="49">
+        <v>2</v>
+      </c>
+      <c r="M35" s="49">
+        <f t="shared" ref="M35" si="14">L35*5</f>
+        <v>10</v>
+      </c>
+      <c r="N35" s="49">
+        <v>20</v>
+      </c>
+      <c r="O35" s="60" t="s">
+        <v>136</v>
+      </c>
+      <c r="P35" s="50">
+        <v>4.8300000000000003E-2</v>
+      </c>
+      <c r="Q35" s="50">
+        <f t="shared" ref="Q35" si="15">P35*N35</f>
+        <v>0.96600000000000008</v>
+      </c>
+      <c r="R35" s="49"/>
+      <c r="S35" s="55"/>
+    </row>
+    <row r="36" spans="1:19" ht="36" x14ac:dyDescent="0.25">
+      <c r="A36" s="1"/>
+      <c r="B36" s="46">
+        <f>ROW(B36) - ROW($B$9)</f>
+        <v>27</v>
+      </c>
+      <c r="C36" s="67" t="s">
+        <v>187</v>
+      </c>
+      <c r="D36" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="E35" s="37" t="s">
+      <c r="E36" s="37" t="s">
         <v>194</v>
       </c>
-      <c r="F35" s="37" t="s">
+      <c r="F36" s="37" t="s">
         <v>135</v>
       </c>
-      <c r="G35" s="37" t="s">
+      <c r="G36" s="37" t="s">
         <v>195</v>
       </c>
-      <c r="H35" s="37" t="s">
+      <c r="H36" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="I35" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="J35" s="37" t="s">
+      <c r="I36" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="J36" s="37" t="s">
         <v>196</v>
       </c>
-      <c r="K35" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="L35" s="37">
-        <v>1</v>
-      </c>
-      <c r="M35" s="37">
-        <f>L35*5</f>
+      <c r="K36" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="L36" s="37">
+        <v>1</v>
+      </c>
+      <c r="M36" s="37">
+        <f>L36*5</f>
         <v>5</v>
       </c>
-      <c r="N35" s="37">
+      <c r="N36" s="37">
         <v>10</v>
       </c>
-      <c r="O35" s="59" t="s">
-        <v>136</v>
-      </c>
-      <c r="P35" s="38">
+      <c r="O36" s="59" t="s">
+        <v>136</v>
+      </c>
+      <c r="P36" s="38">
         <v>6.4600000000000005E-2</v>
       </c>
-      <c r="Q35" s="38">
-        <f>P35*N35</f>
+      <c r="Q36" s="38">
+        <f>P36*N36</f>
         <v>0.64600000000000002</v>
       </c>
-      <c r="R35" s="37"/>
-      <c r="S35" s="55"/>
-    </row>
-    <row r="36" spans="1:19" s="58" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="56"/>
-      <c r="B36" s="46">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-      <c r="C36" s="68" t="s">
-        <v>17</v>
-      </c>
-      <c r="D36" s="49" t="s">
-        <v>34</v>
-      </c>
-      <c r="E36" s="49" t="s">
-        <v>53</v>
-      </c>
-      <c r="F36" s="49" t="s">
-        <v>66</v>
-      </c>
-      <c r="G36" s="49" t="s">
-        <v>83</v>
-      </c>
-      <c r="H36" s="49" t="s">
-        <v>96</v>
-      </c>
-      <c r="I36" s="49" t="s">
-        <v>134</v>
-      </c>
-      <c r="J36" s="49" t="s">
-        <v>114</v>
-      </c>
-      <c r="K36" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="L36" s="49">
-        <v>1</v>
-      </c>
-      <c r="M36" s="49">
-        <f t="shared" ref="M36" si="16">L36*5</f>
-        <v>5</v>
-      </c>
-      <c r="N36" s="49">
-        <v>10</v>
-      </c>
-      <c r="O36" s="60" t="s">
-        <v>136</v>
-      </c>
-      <c r="P36" s="50">
-        <v>0.2079</v>
-      </c>
-      <c r="Q36" s="50">
-        <f t="shared" ref="Q36" si="17">P36*N36</f>
-        <v>2.0790000000000002</v>
-      </c>
-      <c r="R36" s="49"/>
+      <c r="R36" s="37"/>
       <c r="S36" s="55"/>
     </row>
     <row r="37" spans="1:19" s="58" customFormat="1" x14ac:dyDescent="0.25">
@@ -5989,28 +6061,28 @@
         <v>28</v>
       </c>
       <c r="C37" s="68" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D37" s="49" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E37" s="49" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F37" s="49" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G37" s="49" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H37" s="49" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I37" s="49" t="s">
         <v>134</v>
       </c>
       <c r="J37" s="49" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K37" s="37" t="s">
         <v>134</v>
@@ -6019,112 +6091,114 @@
         <v>1</v>
       </c>
       <c r="M37" s="49">
-        <f t="shared" ref="M37" si="18">L37*5</f>
+        <f t="shared" ref="M37" si="16">L37*5</f>
         <v>5</v>
       </c>
       <c r="N37" s="49">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O37" s="60" t="s">
         <v>136</v>
       </c>
       <c r="P37" s="50">
-        <v>0.54569999999999996</v>
+        <v>0.2079</v>
       </c>
       <c r="Q37" s="50">
-        <f t="shared" ref="Q37" si="19">P37*N37</f>
-        <v>3.2741999999999996</v>
+        <f t="shared" ref="Q37" si="17">P37*N37</f>
+        <v>2.0790000000000002</v>
       </c>
       <c r="R37" s="49"/>
       <c r="S37" s="55"/>
     </row>
-    <row r="38" spans="1:19" s="58" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:19" s="58" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="56"/>
       <c r="B38" s="46">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C38" s="67" t="s">
-        <v>20</v>
-      </c>
-      <c r="D38" s="37" t="s">
-        <v>36</v>
-      </c>
-      <c r="E38" s="37" t="s">
-        <v>55</v>
-      </c>
-      <c r="F38" s="37" t="s">
-        <v>135</v>
-      </c>
-      <c r="G38" s="37" t="s">
-        <v>68</v>
-      </c>
-      <c r="H38" s="37" t="s">
-        <v>98</v>
-      </c>
-      <c r="I38" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="J38" s="37" t="s">
-        <v>116</v>
+      <c r="C38" s="68" t="s">
+        <v>19</v>
+      </c>
+      <c r="D38" s="49" t="s">
+        <v>35</v>
+      </c>
+      <c r="E38" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="F38" s="49" t="s">
+        <v>67</v>
+      </c>
+      <c r="G38" s="49" t="s">
+        <v>84</v>
+      </c>
+      <c r="H38" s="49" t="s">
+        <v>97</v>
+      </c>
+      <c r="I38" s="49" t="s">
+        <v>134</v>
+      </c>
+      <c r="J38" s="49" t="s">
+        <v>115</v>
       </c>
       <c r="K38" s="37" t="s">
         <v>134</v>
       </c>
-      <c r="L38" s="37">
-        <v>1</v>
-      </c>
-      <c r="M38" s="37">
-        <f>L38*5</f>
+      <c r="L38" s="49">
+        <v>1</v>
+      </c>
+      <c r="M38" s="49">
+        <f t="shared" ref="M38" si="18">L38*5</f>
         <v>5</v>
       </c>
-      <c r="N38" s="37">
+      <c r="N38" s="49">
         <v>6</v>
       </c>
-      <c r="O38" s="59" t="s">
-        <v>136</v>
-      </c>
-      <c r="P38" s="38">
-        <v>2.8589000000000002</v>
-      </c>
-      <c r="Q38" s="38">
-        <f>P38*N38</f>
-        <v>17.153400000000001</v>
-      </c>
-      <c r="R38" s="37"/>
-      <c r="S38" s="39"/>
-    </row>
-    <row r="39" spans="1:19" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="O38" s="60" t="s">
+        <v>136</v>
+      </c>
+      <c r="P38" s="50">
+        <v>0.54569999999999996</v>
+      </c>
+      <c r="Q38" s="50">
+        <f t="shared" ref="Q38" si="19">P38*N38</f>
+        <v>3.2741999999999996</v>
+      </c>
+      <c r="R38" s="49"/>
+      <c r="S38" s="55"/>
+    </row>
+    <row r="39" spans="1:19" s="58" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="56"/>
       <c r="B39" s="46">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C39" s="67" t="s">
-        <v>144</v>
+        <v>20</v>
       </c>
       <c r="D39" s="37" t="s">
-        <v>143</v>
+        <v>36</v>
       </c>
       <c r="E39" s="37" t="s">
-        <v>225</v>
+        <v>55</v>
       </c>
       <c r="F39" s="37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G39" s="37" t="s">
-        <v>134</v>
+        <v>68</v>
       </c>
       <c r="H39" s="37" t="s">
-        <v>134</v>
+        <v>98</v>
       </c>
       <c r="I39" s="37" t="s">
         <v>134</v>
       </c>
       <c r="J39" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="K39" s="37"/>
+        <v>116</v>
+      </c>
+      <c r="K39" s="37" t="s">
+        <v>134</v>
+      </c>
       <c r="L39" s="37">
         <v>1</v>
       </c>
@@ -6133,17 +6207,17 @@
         <v>5</v>
       </c>
       <c r="N39" s="37">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O39" s="59" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="P39" s="38">
-        <v>4.67</v>
+        <v>2.8589000000000002</v>
       </c>
       <c r="Q39" s="38">
         <f>P39*N39</f>
-        <v>23.35</v>
+        <v>17.153400000000001</v>
       </c>
       <c r="R39" s="37"/>
       <c r="S39" s="39"/>
@@ -6155,13 +6229,13 @@
         <v>31</v>
       </c>
       <c r="C40" s="67" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D40" s="37" t="s">
         <v>143</v>
       </c>
       <c r="E40" s="37" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F40" s="37" t="s">
         <v>134</v>
@@ -6187,80 +6261,134 @@
         <v>5</v>
       </c>
       <c r="N40" s="37">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O40" s="59" t="s">
         <v>147</v>
       </c>
       <c r="P40" s="38">
-        <v>0.35</v>
-      </c>
-      <c r="Q40" s="71">
+        <v>4.67</v>
+      </c>
+      <c r="Q40" s="38">
         <f>P40*N40</f>
-        <v>0.35</v>
+        <v>23.35</v>
       </c>
       <c r="R40" s="37"/>
       <c r="S40" s="39"/>
     </row>
-    <row r="41" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="1"/>
-      <c r="B41" s="40"/>
-      <c r="C41" s="41"/>
-      <c r="D41" s="42"/>
-      <c r="E41" s="43"/>
-      <c r="F41" s="44"/>
-      <c r="G41" s="45"/>
-      <c r="H41" s="44"/>
-      <c r="I41" s="45"/>
-      <c r="J41" s="44"/>
-      <c r="K41" s="45"/>
-      <c r="L41" s="45"/>
-      <c r="M41" s="45"/>
-      <c r="N41" s="95" t="s">
+    <row r="41" spans="1:19" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="56"/>
+      <c r="B41" s="46">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="C41" s="67" t="s">
+        <v>145</v>
+      </c>
+      <c r="D41" s="37" t="s">
+        <v>143</v>
+      </c>
+      <c r="E41" s="37" t="s">
+        <v>226</v>
+      </c>
+      <c r="F41" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="G41" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="H41" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="I41" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="J41" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="K41" s="37"/>
+      <c r="L41" s="37">
+        <v>1</v>
+      </c>
+      <c r="M41" s="37">
+        <f>L41*5</f>
         <v>5</v>
       </c>
-      <c r="O41" s="96"/>
-      <c r="P41" s="96"/>
-      <c r="Q41" s="47">
-        <f>SUM(Q10:Q40)</f>
-        <v>64.005400000000009</v>
-      </c>
-      <c r="R41" s="97"/>
-      <c r="S41" s="98"/>
+      <c r="N41" s="37">
+        <v>1</v>
+      </c>
+      <c r="O41" s="59" t="s">
+        <v>147</v>
+      </c>
+      <c r="P41" s="38">
+        <v>0.35</v>
+      </c>
+      <c r="Q41" s="71">
+        <f>P41*N41</f>
+        <v>0.35</v>
+      </c>
+      <c r="R41" s="37"/>
+      <c r="S41" s="39"/>
     </row>
     <row r="42" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
-      <c r="B42" s="25"/>
-      <c r="C42" s="36"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="10"/>
-      <c r="F42" s="10"/>
-      <c r="G42" s="10"/>
-      <c r="H42" s="10"/>
-      <c r="I42" s="10"/>
-      <c r="J42" s="10"/>
-      <c r="K42" s="10"/>
-      <c r="L42" s="10"/>
-      <c r="M42" s="10"/>
+      <c r="B42" s="40"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="42"/>
+      <c r="E42" s="43"/>
+      <c r="F42" s="44"/>
+      <c r="G42" s="45"/>
+      <c r="H42" s="44"/>
+      <c r="I42" s="45"/>
+      <c r="J42" s="44"/>
+      <c r="K42" s="45"/>
+      <c r="L42" s="45"/>
+      <c r="M42" s="45"/>
       <c r="N42" s="95" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O42" s="96"/>
       <c r="P42" s="96"/>
-      <c r="Q42" s="48">
-        <f>Q41/5</f>
-        <v>12.801080000000002</v>
-      </c>
-      <c r="R42" s="99"/>
-      <c r="S42" s="100"/>
+      <c r="Q42" s="47">
+        <f>SUM(Q10:Q41)</f>
+        <v>64.105400000000003</v>
+      </c>
+      <c r="R42" s="97"/>
+      <c r="S42" s="98"/>
+    </row>
+    <row r="43" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="1"/>
+      <c r="B43" s="25"/>
+      <c r="C43" s="36"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="10"/>
+      <c r="M43" s="10"/>
+      <c r="N43" s="95" t="s">
+        <v>6</v>
+      </c>
+      <c r="O43" s="96"/>
+      <c r="P43" s="96"/>
+      <c r="Q43" s="48">
+        <f>Q42/5</f>
+        <v>12.82108</v>
+      </c>
+      <c r="R43" s="99"/>
+      <c r="S43" s="100"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
-    <mergeCell ref="N41:P41"/>
-    <mergeCell ref="R41:S42"/>
     <mergeCell ref="N42:P42"/>
+    <mergeCell ref="R42:S43"/>
+    <mergeCell ref="N43:P43"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O11" r:id="rId1"/>
@@ -6277,33 +6405,34 @@
     <hyperlink ref="O30" r:id="rId12"/>
     <hyperlink ref="O26" r:id="rId13"/>
     <hyperlink ref="O31" r:id="rId14"/>
-    <hyperlink ref="O36" r:id="rId15"/>
-    <hyperlink ref="O37" r:id="rId16"/>
-    <hyperlink ref="O38" r:id="rId17"/>
+    <hyperlink ref="O37" r:id="rId15"/>
+    <hyperlink ref="O38" r:id="rId16"/>
+    <hyperlink ref="O39" r:id="rId17"/>
     <hyperlink ref="O10" r:id="rId18"/>
     <hyperlink ref="O14" r:id="rId19"/>
     <hyperlink ref="O23" r:id="rId20"/>
     <hyperlink ref="O25" r:id="rId21"/>
     <hyperlink ref="O29" r:id="rId22"/>
     <hyperlink ref="O32" r:id="rId23"/>
-    <hyperlink ref="O33" r:id="rId24"/>
-    <hyperlink ref="O34" r:id="rId25"/>
-    <hyperlink ref="O35" r:id="rId26"/>
+    <hyperlink ref="O34" r:id="rId24"/>
+    <hyperlink ref="O35" r:id="rId25"/>
+    <hyperlink ref="O36" r:id="rId26"/>
     <hyperlink ref="O17" r:id="rId27"/>
     <hyperlink ref="O28" r:id="rId28"/>
     <hyperlink ref="O24" r:id="rId29"/>
-    <hyperlink ref="O39" r:id="rId30"/>
-    <hyperlink ref="O40" r:id="rId31"/>
+    <hyperlink ref="O40" r:id="rId30"/>
+    <hyperlink ref="O41" r:id="rId31"/>
+    <hyperlink ref="O33" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId32"/>
-  <drawing r:id="rId33"/>
+  <pageSetup orientation="portrait" r:id="rId33"/>
+  <drawing r:id="rId34"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S42"/>
+  <dimension ref="A1:S43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
@@ -6681,7 +6810,7 @@
     <row r="12" spans="1:19" s="58" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="56"/>
       <c r="B12" s="46">
-        <f t="shared" ref="B12:B40" si="0">ROW(B12) - ROW($B$9)</f>
+        <f t="shared" ref="B12:B41" si="0">ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
       <c r="C12" s="67" t="s">
@@ -6715,7 +6844,7 @@
         <v>2</v>
       </c>
       <c r="M12" s="37">
-        <f t="shared" ref="M12:M40" si="1">L12*50</f>
+        <f t="shared" ref="M12:M41" si="1">L12*50</f>
         <v>100</v>
       </c>
       <c r="N12" s="37">
@@ -7796,7 +7925,7 @@
     <row r="32" spans="1:19" s="58" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="56"/>
       <c r="B32" s="72">
-        <f t="shared" ref="B32" si="8">ROW(B32) - ROW($B$9)</f>
+        <f t="shared" ref="B32:B33" si="8">ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
       <c r="C32" s="87" t="s">
@@ -7850,259 +7979,259 @@
       </c>
       <c r="S32" s="94"/>
     </row>
-    <row r="33" spans="1:19" s="58" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33" s="56"/>
       <c r="B33" s="46">
-        <f>ROW(B33) - ROW($B$9)</f>
+        <f t="shared" si="8"/>
         <v>24</v>
       </c>
-      <c r="C33" s="68" t="s">
+      <c r="C33" s="67" t="s">
+        <v>18</v>
+      </c>
+      <c r="D33" s="49" t="s">
+        <v>228</v>
+      </c>
+      <c r="E33" s="85" t="s">
+        <v>229</v>
+      </c>
+      <c r="F33" s="49" t="s">
+        <v>65</v>
+      </c>
+      <c r="G33" s="85" t="s">
+        <v>230</v>
+      </c>
+      <c r="H33" s="49" t="s">
+        <v>86</v>
+      </c>
+      <c r="I33" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="J33" s="37" t="s">
+        <v>231</v>
+      </c>
+      <c r="K33" s="37" t="s">
+        <v>232</v>
+      </c>
+      <c r="L33" s="37">
+        <v>1</v>
+      </c>
+      <c r="M33" s="37">
+        <f>L33*50</f>
+        <v>50</v>
+      </c>
+      <c r="N33" s="37">
+        <v>100</v>
+      </c>
+      <c r="O33" s="59" t="s">
+        <v>136</v>
+      </c>
+      <c r="P33" s="38">
+        <v>1E-3</v>
+      </c>
+      <c r="Q33" s="50">
+        <f>P33*N33</f>
+        <v>0.1</v>
+      </c>
+      <c r="R33" s="76"/>
+      <c r="S33" s="55"/>
+    </row>
+    <row r="34" spans="1:19" s="58" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A34" s="56"/>
+      <c r="B34" s="46">
+        <f>ROW(B34) - ROW($B$9)</f>
+        <v>25</v>
+      </c>
+      <c r="C34" s="68" t="s">
         <v>187</v>
       </c>
-      <c r="D33" s="37" t="s">
+      <c r="D34" s="37" t="s">
         <v>33</v>
       </c>
-      <c r="E33" s="37" t="s">
+      <c r="E34" s="37" t="s">
         <v>185</v>
       </c>
-      <c r="F33" s="37" t="s">
+      <c r="F34" s="37" t="s">
         <v>135</v>
       </c>
-      <c r="G33" s="37" t="s">
+      <c r="G34" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="H33" s="37" t="s">
+      <c r="H34" s="37" t="s">
         <v>184</v>
       </c>
-      <c r="I33" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="J33" s="37" t="s">
+      <c r="I34" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="J34" s="37" t="s">
         <v>197</v>
       </c>
-      <c r="K33" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="L33" s="37">
-        <v>1</v>
-      </c>
-      <c r="M33" s="37">
+      <c r="K34" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="L34" s="37">
+        <v>1</v>
+      </c>
+      <c r="M34" s="37">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="N33" s="37">
+      <c r="N34" s="37">
         <v>55</v>
       </c>
-      <c r="O33" s="59" t="s">
-        <v>136</v>
-      </c>
-      <c r="P33" s="38">
+      <c r="O34" s="59" t="s">
+        <v>136</v>
+      </c>
+      <c r="P34" s="38">
         <v>0.1336</v>
       </c>
-      <c r="Q33" s="38">
-        <f>P33*N33</f>
+      <c r="Q34" s="38">
+        <f>P34*N34</f>
         <v>7.3479999999999999</v>
       </c>
-      <c r="R33" s="37"/>
-      <c r="S33" s="55"/>
-    </row>
-    <row r="34" spans="1:19" s="58" customFormat="1" ht="36" x14ac:dyDescent="0.25">
-      <c r="A34" s="56"/>
-      <c r="B34" s="72">
-        <f t="shared" ref="B34" si="9">ROW(B34) - ROW($B$9)</f>
-        <v>25</v>
-      </c>
-      <c r="C34" s="68" t="s">
+      <c r="R34" s="37"/>
+      <c r="S34" s="55"/>
+    </row>
+    <row r="35" spans="1:19" s="58" customFormat="1" ht="36" x14ac:dyDescent="0.25">
+      <c r="A35" s="56"/>
+      <c r="B35" s="72">
+        <f t="shared" ref="B35" si="9">ROW(B35) - ROW($B$9)</f>
+        <v>26</v>
+      </c>
+      <c r="C35" s="68" t="s">
         <v>187</v>
       </c>
-      <c r="D34" s="49" t="s">
+      <c r="D35" s="49" t="s">
         <v>188</v>
       </c>
-      <c r="E34" s="49" t="s">
+      <c r="E35" s="49" t="s">
         <v>189</v>
       </c>
-      <c r="F34" s="49" t="s">
+      <c r="F35" s="49" t="s">
         <v>135</v>
       </c>
-      <c r="G34" s="49" t="s">
+      <c r="G35" s="49" t="s">
         <v>190</v>
       </c>
-      <c r="H34" s="49" t="s">
+      <c r="H35" s="49" t="s">
         <v>191</v>
       </c>
-      <c r="I34" s="49" t="s">
-        <v>134</v>
-      </c>
-      <c r="J34" s="49" t="s">
+      <c r="I35" s="49" t="s">
+        <v>134</v>
+      </c>
+      <c r="J35" s="49" t="s">
         <v>192</v>
       </c>
-      <c r="K34" s="49" t="s">
-        <v>134</v>
-      </c>
-      <c r="L34" s="49">
+      <c r="K35" s="49" t="s">
+        <v>134</v>
+      </c>
+      <c r="L35" s="49">
         <v>2</v>
       </c>
-      <c r="M34" s="37">
+      <c r="M35" s="37">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="N34" s="49">
+      <c r="N35" s="49">
         <v>110</v>
       </c>
-      <c r="O34" s="60" t="s">
-        <v>136</v>
-      </c>
-      <c r="P34" s="50">
+      <c r="O35" s="60" t="s">
+        <v>136</v>
+      </c>
+      <c r="P35" s="50">
         <v>4.1399999999999999E-2</v>
       </c>
-      <c r="Q34" s="50">
-        <f t="shared" ref="Q34" si="10">P34*N34</f>
+      <c r="Q35" s="50">
+        <f t="shared" ref="Q35" si="10">P35*N35</f>
         <v>4.5540000000000003</v>
       </c>
-      <c r="R34" s="49"/>
-      <c r="S34" s="55"/>
-    </row>
-    <row r="35" spans="1:19" s="58" customFormat="1" ht="36" x14ac:dyDescent="0.25">
-      <c r="A35" s="56"/>
-      <c r="B35" s="46">
-        <f>ROW(B35) - ROW($B$9)</f>
-        <v>26</v>
-      </c>
-      <c r="C35" s="67" t="s">
-        <v>187</v>
-      </c>
-      <c r="D35" s="37" t="s">
-        <v>193</v>
-      </c>
-      <c r="E35" s="37" t="s">
-        <v>194</v>
-      </c>
-      <c r="F35" s="37" t="s">
-        <v>135</v>
-      </c>
-      <c r="G35" s="37" t="s">
-        <v>195</v>
-      </c>
-      <c r="H35" s="37" t="s">
-        <v>94</v>
-      </c>
-      <c r="I35" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="J35" s="37" t="s">
-        <v>196</v>
-      </c>
-      <c r="K35" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="L35" s="37">
-        <v>1</v>
-      </c>
-      <c r="M35" s="37">
-        <f t="shared" si="1"/>
-        <v>50</v>
-      </c>
-      <c r="N35" s="37">
-        <v>60</v>
-      </c>
-      <c r="O35" s="59" t="s">
-        <v>136</v>
-      </c>
-      <c r="P35" s="38">
-        <v>6.4600000000000005E-2</v>
-      </c>
-      <c r="Q35" s="38">
-        <f>P35*N35</f>
-        <v>3.8760000000000003</v>
-      </c>
-      <c r="R35" s="37"/>
+      <c r="R35" s="49"/>
       <c r="S35" s="55"/>
     </row>
-    <row r="36" spans="1:19" s="58" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" s="58" customFormat="1" ht="36" x14ac:dyDescent="0.25">
       <c r="A36" s="56"/>
       <c r="B36" s="46">
-        <f t="shared" si="0"/>
+        <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
-      <c r="C36" s="68" t="s">
-        <v>17</v>
-      </c>
-      <c r="D36" s="49" t="s">
-        <v>34</v>
-      </c>
-      <c r="E36" s="49" t="s">
-        <v>53</v>
-      </c>
-      <c r="F36" s="49" t="s">
-        <v>66</v>
-      </c>
-      <c r="G36" s="49" t="s">
-        <v>83</v>
-      </c>
-      <c r="H36" s="49" t="s">
-        <v>96</v>
-      </c>
-      <c r="I36" s="49" t="s">
-        <v>134</v>
-      </c>
-      <c r="J36" s="49" t="s">
-        <v>114</v>
+      <c r="C36" s="67" t="s">
+        <v>187</v>
+      </c>
+      <c r="D36" s="37" t="s">
+        <v>193</v>
+      </c>
+      <c r="E36" s="37" t="s">
+        <v>194</v>
+      </c>
+      <c r="F36" s="37" t="s">
+        <v>135</v>
+      </c>
+      <c r="G36" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="H36" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="I36" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="J36" s="37" t="s">
+        <v>196</v>
       </c>
       <c r="K36" s="37" t="s">
         <v>134</v>
       </c>
-      <c r="L36" s="49">
+      <c r="L36" s="37">
         <v>1</v>
       </c>
       <c r="M36" s="37">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="N36" s="49">
-        <v>55</v>
-      </c>
-      <c r="O36" s="60" t="s">
-        <v>136</v>
-      </c>
-      <c r="P36" s="50">
-        <v>0.14460000000000001</v>
-      </c>
-      <c r="Q36" s="50">
-        <f t="shared" ref="Q36:Q37" si="11">P36*N36</f>
-        <v>7.9530000000000003</v>
-      </c>
-      <c r="R36" s="49"/>
+      <c r="N36" s="37">
+        <v>60</v>
+      </c>
+      <c r="O36" s="59" t="s">
+        <v>136</v>
+      </c>
+      <c r="P36" s="38">
+        <v>6.4600000000000005E-2</v>
+      </c>
+      <c r="Q36" s="38">
+        <f>P36*N36</f>
+        <v>3.8760000000000003</v>
+      </c>
+      <c r="R36" s="37"/>
       <c r="S36" s="55"/>
     </row>
-    <row r="37" spans="1:19" s="58" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" s="58" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="56"/>
       <c r="B37" s="46">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C37" s="68" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D37" s="49" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E37" s="49" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F37" s="49" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G37" s="49" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H37" s="49" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I37" s="49" t="s">
         <v>134</v>
       </c>
       <c r="J37" s="49" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K37" s="37" t="s">
         <v>134</v>
@@ -8115,108 +8244,110 @@
         <v>50</v>
       </c>
       <c r="N37" s="49">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="O37" s="60" t="s">
         <v>136</v>
       </c>
       <c r="P37" s="50">
-        <v>0.4073</v>
+        <v>0.14460000000000001</v>
       </c>
       <c r="Q37" s="50">
-        <f t="shared" si="11"/>
-        <v>21.179600000000001</v>
+        <f t="shared" ref="Q37:Q38" si="11">P37*N37</f>
+        <v>7.9530000000000003</v>
       </c>
       <c r="R37" s="49"/>
       <c r="S37" s="55"/>
     </row>
-    <row r="38" spans="1:19" s="58" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:19" s="58" customFormat="1" ht="24" x14ac:dyDescent="0.25">
       <c r="A38" s="56"/>
       <c r="B38" s="46">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C38" s="67" t="s">
-        <v>20</v>
-      </c>
-      <c r="D38" s="37" t="s">
-        <v>36</v>
-      </c>
-      <c r="E38" s="37" t="s">
-        <v>55</v>
-      </c>
-      <c r="F38" s="37" t="s">
-        <v>135</v>
-      </c>
-      <c r="G38" s="37" t="s">
-        <v>68</v>
-      </c>
-      <c r="H38" s="37" t="s">
-        <v>98</v>
-      </c>
-      <c r="I38" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="J38" s="37" t="s">
-        <v>116</v>
+      <c r="C38" s="68" t="s">
+        <v>19</v>
+      </c>
+      <c r="D38" s="49" t="s">
+        <v>35</v>
+      </c>
+      <c r="E38" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="F38" s="49" t="s">
+        <v>67</v>
+      </c>
+      <c r="G38" s="49" t="s">
+        <v>84</v>
+      </c>
+      <c r="H38" s="49" t="s">
+        <v>97</v>
+      </c>
+      <c r="I38" s="49" t="s">
+        <v>134</v>
+      </c>
+      <c r="J38" s="49" t="s">
+        <v>115</v>
       </c>
       <c r="K38" s="37" t="s">
         <v>134</v>
       </c>
-      <c r="L38" s="37">
+      <c r="L38" s="49">
         <v>1</v>
       </c>
       <c r="M38" s="37">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="N38" s="37">
+      <c r="N38" s="49">
         <v>52</v>
       </c>
-      <c r="O38" s="59" t="s">
-        <v>136</v>
-      </c>
-      <c r="P38" s="38">
-        <v>2.7953000000000001</v>
-      </c>
-      <c r="Q38" s="38">
-        <f>P38*N38</f>
-        <v>145.35560000000001</v>
-      </c>
-      <c r="R38" s="37"/>
-      <c r="S38" s="39"/>
-    </row>
-    <row r="39" spans="1:19" s="58" customFormat="1" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="O38" s="60" t="s">
+        <v>136</v>
+      </c>
+      <c r="P38" s="50">
+        <v>0.4073</v>
+      </c>
+      <c r="Q38" s="50">
+        <f t="shared" si="11"/>
+        <v>21.179600000000001</v>
+      </c>
+      <c r="R38" s="49"/>
+      <c r="S38" s="55"/>
+    </row>
+    <row r="39" spans="1:19" s="58" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="56"/>
       <c r="B39" s="46">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C39" s="67" t="s">
-        <v>144</v>
+        <v>20</v>
       </c>
       <c r="D39" s="37" t="s">
-        <v>143</v>
+        <v>36</v>
       </c>
       <c r="E39" s="37" t="s">
-        <v>225</v>
+        <v>55</v>
       </c>
       <c r="F39" s="37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G39" s="37" t="s">
-        <v>134</v>
+        <v>68</v>
       </c>
       <c r="H39" s="37" t="s">
-        <v>134</v>
+        <v>98</v>
       </c>
       <c r="I39" s="37" t="s">
         <v>134</v>
       </c>
       <c r="J39" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="K39" s="37"/>
+        <v>116</v>
+      </c>
+      <c r="K39" s="37" t="s">
+        <v>134</v>
+      </c>
       <c r="L39" s="37">
         <v>1</v>
       </c>
@@ -8225,17 +8356,17 @@
         <v>50</v>
       </c>
       <c r="N39" s="37">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="O39" s="59" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="P39" s="38">
-        <v>4.67</v>
+        <v>2.7953000000000001</v>
       </c>
       <c r="Q39" s="38">
         <f>P39*N39</f>
-        <v>233.5</v>
+        <v>145.35560000000001</v>
       </c>
       <c r="R39" s="37"/>
       <c r="S39" s="39"/>
@@ -8247,13 +8378,13 @@
         <v>31</v>
       </c>
       <c r="C40" s="67" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D40" s="37" t="s">
         <v>143</v>
       </c>
       <c r="E40" s="37" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F40" s="37" t="s">
         <v>134</v>
@@ -8285,74 +8416,128 @@
         <v>147</v>
       </c>
       <c r="P40" s="38">
-        <v>0.35</v>
-      </c>
-      <c r="Q40" s="71">
+        <v>4.67</v>
+      </c>
+      <c r="Q40" s="38">
         <f>P40*N40</f>
-        <v>17.5</v>
+        <v>233.5</v>
       </c>
       <c r="R40" s="37"/>
       <c r="S40" s="39"/>
     </row>
-    <row r="41" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="1"/>
-      <c r="B41" s="40"/>
-      <c r="C41" s="41"/>
-      <c r="D41" s="42"/>
-      <c r="E41" s="43"/>
-      <c r="F41" s="44"/>
-      <c r="G41" s="45"/>
-      <c r="H41" s="44"/>
-      <c r="I41" s="45"/>
-      <c r="J41" s="44"/>
-      <c r="K41" s="45"/>
-      <c r="L41" s="45"/>
-      <c r="M41" s="45"/>
-      <c r="N41" s="95" t="s">
-        <v>5</v>
-      </c>
-      <c r="O41" s="96"/>
-      <c r="P41" s="96"/>
-      <c r="Q41" s="47">
-        <f>SUM(Q10:Q40)</f>
-        <v>515.23210000000006</v>
-      </c>
-      <c r="R41" s="97"/>
-      <c r="S41" s="98"/>
+    <row r="41" spans="1:19" s="58" customFormat="1" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="56"/>
+      <c r="B41" s="46">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="C41" s="67" t="s">
+        <v>145</v>
+      </c>
+      <c r="D41" s="37" t="s">
+        <v>143</v>
+      </c>
+      <c r="E41" s="37" t="s">
+        <v>226</v>
+      </c>
+      <c r="F41" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="G41" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="H41" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="I41" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="J41" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="K41" s="37"/>
+      <c r="L41" s="37">
+        <v>1</v>
+      </c>
+      <c r="M41" s="37">
+        <f t="shared" si="1"/>
+        <v>50</v>
+      </c>
+      <c r="N41" s="37">
+        <v>50</v>
+      </c>
+      <c r="O41" s="59" t="s">
+        <v>147</v>
+      </c>
+      <c r="P41" s="38">
+        <v>0.35</v>
+      </c>
+      <c r="Q41" s="71">
+        <f>P41*N41</f>
+        <v>17.5</v>
+      </c>
+      <c r="R41" s="37"/>
+      <c r="S41" s="39"/>
     </row>
     <row r="42" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
-      <c r="B42" s="25"/>
-      <c r="C42" s="36"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="10"/>
-      <c r="F42" s="10"/>
-      <c r="G42" s="10"/>
-      <c r="H42" s="10"/>
-      <c r="I42" s="10"/>
-      <c r="J42" s="10"/>
-      <c r="K42" s="10"/>
-      <c r="L42" s="10"/>
-      <c r="M42" s="10"/>
+      <c r="B42" s="40"/>
+      <c r="C42" s="41"/>
+      <c r="D42" s="42"/>
+      <c r="E42" s="43"/>
+      <c r="F42" s="44"/>
+      <c r="G42" s="45"/>
+      <c r="H42" s="44"/>
+      <c r="I42" s="45"/>
+      <c r="J42" s="44"/>
+      <c r="K42" s="45"/>
+      <c r="L42" s="45"/>
+      <c r="M42" s="45"/>
       <c r="N42" s="95" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O42" s="96"/>
       <c r="P42" s="96"/>
-      <c r="Q42" s="48">
-        <f>Q41/50</f>
-        <v>10.304642000000001</v>
-      </c>
-      <c r="R42" s="99"/>
-      <c r="S42" s="100"/>
+      <c r="Q42" s="47">
+        <f>SUM(Q10:Q41)</f>
+        <v>515.33210000000008</v>
+      </c>
+      <c r="R42" s="97"/>
+      <c r="S42" s="98"/>
+    </row>
+    <row r="43" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="1"/>
+      <c r="B43" s="25"/>
+      <c r="C43" s="36"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
+      <c r="L43" s="10"/>
+      <c r="M43" s="10"/>
+      <c r="N43" s="95" t="s">
+        <v>6</v>
+      </c>
+      <c r="O43" s="96"/>
+      <c r="P43" s="96"/>
+      <c r="Q43" s="48">
+        <f>Q42/50</f>
+        <v>10.306642000000002</v>
+      </c>
+      <c r="R43" s="99"/>
+      <c r="S43" s="100"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
-    <mergeCell ref="N41:P41"/>
-    <mergeCell ref="R41:S42"/>
     <mergeCell ref="N42:P42"/>
+    <mergeCell ref="R42:S43"/>
+    <mergeCell ref="N43:P43"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O11" r:id="rId1"/>
@@ -8369,27 +8554,28 @@
     <hyperlink ref="O30" r:id="rId12"/>
     <hyperlink ref="O26" r:id="rId13"/>
     <hyperlink ref="O31" r:id="rId14"/>
-    <hyperlink ref="O36" r:id="rId15"/>
-    <hyperlink ref="O37" r:id="rId16"/>
-    <hyperlink ref="O38" r:id="rId17"/>
+    <hyperlink ref="O37" r:id="rId15"/>
+    <hyperlink ref="O38" r:id="rId16"/>
+    <hyperlink ref="O39" r:id="rId17"/>
     <hyperlink ref="O10" r:id="rId18"/>
     <hyperlink ref="O14" r:id="rId19"/>
     <hyperlink ref="O23" r:id="rId20"/>
     <hyperlink ref="O25" r:id="rId21"/>
     <hyperlink ref="O29" r:id="rId22"/>
     <hyperlink ref="O32" r:id="rId23"/>
-    <hyperlink ref="O33" r:id="rId24"/>
-    <hyperlink ref="O34" r:id="rId25"/>
-    <hyperlink ref="O35" r:id="rId26"/>
+    <hyperlink ref="O34" r:id="rId24"/>
+    <hyperlink ref="O35" r:id="rId25"/>
+    <hyperlink ref="O36" r:id="rId26"/>
     <hyperlink ref="O28" r:id="rId27"/>
     <hyperlink ref="O17" r:id="rId28"/>
-    <hyperlink ref="O39" r:id="rId29"/>
-    <hyperlink ref="O40" r:id="rId30"/>
+    <hyperlink ref="O40" r:id="rId29"/>
+    <hyperlink ref="O41" r:id="rId30"/>
     <hyperlink ref="O24" r:id="rId31"/>
+    <hyperlink ref="O33" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId32"/>
-  <drawing r:id="rId33"/>
+  <pageSetup orientation="portrait" r:id="rId33"/>
+  <drawing r:id="rId34"/>
 </worksheet>
 </file>
 

</xml_diff>